<commit_message>
address weirdness with human-animal interface odd character
</commit_message>
<xml_diff>
--- a/data/raw/raw summary cost data.xlsx
+++ b/data/raw/raw summary cost data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stepheaneff/Documents/work/GT/costed-NAPHS/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF701A85-208D-2144-8288-043606ED8B3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DA06D1-6527-C441-8E30-B0ED37A11119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3660" yWindow="760" windowWidth="26580" windowHeight="13180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -331,9 +331,6 @@
     <t>IHR Coordination and National IHR Focal Point Functions</t>
   </si>
   <si>
-    <t>Zoonotic events and the human–animal interface</t>
-  </si>
-  <si>
     <t>Surveillance</t>
   </si>
   <si>
@@ -521,6 +518,9 @@
   </si>
   <si>
     <t>Radiation Events</t>
+  </si>
+  <si>
+    <t>Zoonotic events and the human-animal interface</t>
   </si>
 </sst>
 </file>
@@ -972,7 +972,7 @@
         <v>14</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E4" s="2">
         <v>1547566</v>
@@ -995,7 +995,7 @@
         <v>14</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E5" s="2">
         <v>2165756</v>
@@ -1018,7 +1018,7 @@
         <v>14</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E6" s="1">
         <v>415719</v>
@@ -1041,7 +1041,7 @@
         <v>14</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E7" s="1">
         <v>1059019</v>
@@ -1156,7 +1156,7 @@
         <v>14</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E12" s="1">
         <v>29984</v>
@@ -1202,7 +1202,7 @@
         <v>14</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E14" s="1">
         <v>99881</v>
@@ -1271,7 +1271,7 @@
         <v>14</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E17" s="1">
         <v>898716</v>
@@ -1294,7 +1294,7 @@
         <v>14</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="E18" s="1">
         <v>181294</v>
@@ -1340,7 +1340,7 @@
         <v>14</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="E20" s="1">
         <v>169744</v>
@@ -1708,7 +1708,7 @@
         <v>14</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E36" s="1">
         <v>500000000</v>
@@ -1800,7 +1800,7 @@
         <v>14</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E40" s="1">
         <v>14283000</v>
@@ -2162,7 +2162,7 @@
         <v>14</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E56" s="1">
         <v>12025872</v>
@@ -2245,7 +2245,7 @@
         <v>14</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E60" s="1">
         <v>5492547</v>
@@ -2659,7 +2659,7 @@
         <v>14</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E78" s="2">
         <v>704080</v>
@@ -2751,7 +2751,7 @@
         <v>14</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E82" s="2">
         <v>2394825</v>
@@ -3119,7 +3119,7 @@
         <v>14</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E98" s="3">
         <v>475046.67</v>
@@ -3211,7 +3211,7 @@
         <v>14</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E102" s="3">
         <v>2238841.7799999998</v>
@@ -3303,7 +3303,7 @@
         <v>14</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E106" s="2">
         <v>3965056</v>
@@ -3326,7 +3326,7 @@
         <v>14</v>
       </c>
       <c r="D107" s="4" t="s">
-        <v>103</v>
+        <v>166</v>
       </c>
       <c r="E107" s="2">
         <v>2184075</v>
@@ -3349,7 +3349,7 @@
         <v>14</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E108" s="2">
         <v>2622819</v>
@@ -3372,7 +3372,7 @@
         <v>14</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E109" s="2">
         <v>6507557</v>
@@ -3441,7 +3441,7 @@
         <v>14</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E112" s="2">
         <v>21871396</v>
@@ -3487,7 +3487,7 @@
         <v>14</v>
       </c>
       <c r="D114" s="4" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E114" s="2">
         <v>37262878</v>
@@ -3533,7 +3533,7 @@
         <v>14</v>
       </c>
       <c r="D116" s="4" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E116" s="2">
         <v>571606</v>
@@ -3556,7 +3556,7 @@
         <v>14</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E117" s="2">
         <v>6900995</v>
@@ -3579,7 +3579,7 @@
         <v>14</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E118" s="2">
         <v>606221</v>
@@ -3602,7 +3602,7 @@
         <v>14</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E119" s="2">
         <v>1711218</v>
@@ -3671,7 +3671,7 @@
         <v>14</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E122" s="2">
         <v>662055</v>
@@ -3688,7 +3688,7 @@
         <v>122</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C123" s="1" t="s">
         <v>35</v>
@@ -3703,7 +3703,7 @@
         <v>78</v>
       </c>
       <c r="G123" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.2">
@@ -3711,7 +3711,7 @@
         <v>123</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C124" s="1" t="s">
         <v>14</v>
@@ -3726,7 +3726,7 @@
         <v>78</v>
       </c>
       <c r="G124" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.2">
@@ -3734,7 +3734,7 @@
         <v>124</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C125" s="1" t="s">
         <v>14</v>
@@ -3749,7 +3749,7 @@
         <v>78</v>
       </c>
       <c r="G125" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.2">
@@ -3757,7 +3757,7 @@
         <v>125</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C126" s="1" t="s">
         <v>14</v>
@@ -3772,7 +3772,7 @@
         <v>78</v>
       </c>
       <c r="G126" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.2">
@@ -3780,7 +3780,7 @@
         <v>126</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C127" s="1" t="s">
         <v>14</v>
@@ -3795,7 +3795,7 @@
         <v>78</v>
       </c>
       <c r="G127" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.2">
@@ -3803,7 +3803,7 @@
         <v>127</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C128" s="1" t="s">
         <v>14</v>
@@ -3818,7 +3818,7 @@
         <v>78</v>
       </c>
       <c r="G128" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.2">
@@ -3826,7 +3826,7 @@
         <v>128</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C129" s="1" t="s">
         <v>14</v>
@@ -3841,7 +3841,7 @@
         <v>78</v>
       </c>
       <c r="G129" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.2">
@@ -3849,7 +3849,7 @@
         <v>129</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C130" s="1" t="s">
         <v>14</v>
@@ -3864,7 +3864,7 @@
         <v>78</v>
       </c>
       <c r="G130" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.2">
@@ -3872,7 +3872,7 @@
         <v>130</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C131" s="1" t="s">
         <v>14</v>
@@ -3887,7 +3887,7 @@
         <v>78</v>
       </c>
       <c r="G131" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.2">
@@ -3895,7 +3895,7 @@
         <v>131</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C132" s="1" t="s">
         <v>14</v>
@@ -3910,7 +3910,7 @@
         <v>78</v>
       </c>
       <c r="G132" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="133" spans="1:7" x14ac:dyDescent="0.2">
@@ -3918,7 +3918,7 @@
         <v>132</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C133" s="1" t="s">
         <v>14</v>
@@ -3933,7 +3933,7 @@
         <v>78</v>
       </c>
       <c r="G133" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="134" spans="1:7" x14ac:dyDescent="0.2">
@@ -3941,7 +3941,7 @@
         <v>133</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C134" s="1" t="s">
         <v>14</v>
@@ -3956,7 +3956,7 @@
         <v>78</v>
       </c>
       <c r="G134" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="135" spans="1:7" x14ac:dyDescent="0.2">
@@ -3964,7 +3964,7 @@
         <v>134</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C135" s="1" t="s">
         <v>14</v>
@@ -3979,7 +3979,7 @@
         <v>78</v>
       </c>
       <c r="G135" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="136" spans="1:7" x14ac:dyDescent="0.2">
@@ -3987,7 +3987,7 @@
         <v>135</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C136" s="1" t="s">
         <v>14</v>
@@ -4002,7 +4002,7 @@
         <v>78</v>
       </c>
       <c r="G136" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="137" spans="1:7" x14ac:dyDescent="0.2">
@@ -4010,7 +4010,7 @@
         <v>136</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C137" s="1" t="s">
         <v>14</v>
@@ -4025,7 +4025,7 @@
         <v>78</v>
       </c>
       <c r="G137" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="138" spans="1:7" x14ac:dyDescent="0.2">
@@ -4033,13 +4033,13 @@
         <v>137</v>
       </c>
       <c r="B138" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D138" s="1" t="s">
         <v>110</v>
-      </c>
-      <c r="C138" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D138" s="1" t="s">
-        <v>111</v>
       </c>
       <c r="E138" s="2">
         <v>174708</v>
@@ -4048,7 +4048,7 @@
         <v>78</v>
       </c>
       <c r="G138" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="139" spans="1:7" x14ac:dyDescent="0.2">
@@ -4056,7 +4056,7 @@
         <v>138</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C139" s="1" t="s">
         <v>14</v>
@@ -4071,7 +4071,7 @@
         <v>78</v>
       </c>
       <c r="G139" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="140" spans="1:7" x14ac:dyDescent="0.2">
@@ -4079,7 +4079,7 @@
         <v>139</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C140" s="1" t="s">
         <v>14</v>
@@ -4094,7 +4094,7 @@
         <v>78</v>
       </c>
       <c r="G140" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="141" spans="1:7" x14ac:dyDescent="0.2">
@@ -4102,7 +4102,7 @@
         <v>140</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C141" s="1" t="s">
         <v>14</v>
@@ -4117,7 +4117,7 @@
         <v>78</v>
       </c>
       <c r="G141" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="142" spans="1:7" x14ac:dyDescent="0.2">
@@ -4125,13 +4125,13 @@
         <v>141</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C142" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D142" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E142" s="2">
         <v>5421278</v>
@@ -4140,7 +4140,7 @@
         <v>78</v>
       </c>
       <c r="G142" s="1" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="143" spans="1:7" x14ac:dyDescent="0.2">
@@ -4148,7 +4148,7 @@
         <v>142</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C143" s="1" t="s">
         <v>35</v>
@@ -4163,7 +4163,7 @@
         <v>4</v>
       </c>
       <c r="G143" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="144" spans="1:7" x14ac:dyDescent="0.2">
@@ -4171,7 +4171,7 @@
         <v>143</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C144" s="1" t="s">
         <v>14</v>
@@ -4186,7 +4186,7 @@
         <v>4</v>
       </c>
       <c r="G144" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="145" spans="1:7" x14ac:dyDescent="0.2">
@@ -4194,7 +4194,7 @@
         <v>144</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C145" s="1" t="s">
         <v>14</v>
@@ -4209,7 +4209,7 @@
         <v>4</v>
       </c>
       <c r="G145" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="146" spans="1:7" x14ac:dyDescent="0.2">
@@ -4217,13 +4217,13 @@
         <v>145</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C146" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E146" s="2">
         <v>1922152</v>
@@ -4232,7 +4232,7 @@
         <v>4</v>
       </c>
       <c r="G146" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="147" spans="1:7" x14ac:dyDescent="0.2">
@@ -4240,13 +4240,13 @@
         <v>146</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C147" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D147" s="1" t="s">
-        <v>103</v>
+        <v>166</v>
       </c>
       <c r="E147" s="2">
         <v>1468086</v>
@@ -4255,7 +4255,7 @@
         <v>4</v>
       </c>
       <c r="G147" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="148" spans="1:7" x14ac:dyDescent="0.2">
@@ -4263,13 +4263,13 @@
         <v>147</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C148" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D148" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E148" s="2">
         <v>613709</v>
@@ -4278,7 +4278,7 @@
         <v>4</v>
       </c>
       <c r="G148" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="149" spans="1:7" x14ac:dyDescent="0.2">
@@ -4286,13 +4286,13 @@
         <v>148</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C149" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E149" s="2">
         <v>1518082</v>
@@ -4301,7 +4301,7 @@
         <v>4</v>
       </c>
       <c r="G149" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="150" spans="1:7" x14ac:dyDescent="0.2">
@@ -4309,7 +4309,7 @@
         <v>149</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C150" s="1" t="s">
         <v>14</v>
@@ -4324,7 +4324,7 @@
         <v>4</v>
       </c>
       <c r="G150" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="151" spans="1:7" x14ac:dyDescent="0.2">
@@ -4332,7 +4332,7 @@
         <v>150</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C151" s="1" t="s">
         <v>14</v>
@@ -4347,7 +4347,7 @@
         <v>4</v>
       </c>
       <c r="G151" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="152" spans="1:7" x14ac:dyDescent="0.2">
@@ -4355,7 +4355,7 @@
         <v>151</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C152" s="1" t="s">
         <v>14</v>
@@ -4370,7 +4370,7 @@
         <v>4</v>
       </c>
       <c r="G152" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="153" spans="1:7" x14ac:dyDescent="0.2">
@@ -4378,7 +4378,7 @@
         <v>152</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C153" s="1" t="s">
         <v>14</v>
@@ -4393,7 +4393,7 @@
         <v>4</v>
       </c>
       <c r="G153" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="154" spans="1:7" x14ac:dyDescent="0.2">
@@ -4401,13 +4401,13 @@
         <v>153</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C154" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E154" s="2">
         <v>118398</v>
@@ -4416,7 +4416,7 @@
         <v>4</v>
       </c>
       <c r="G154" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="155" spans="1:7" x14ac:dyDescent="0.2">
@@ -4424,7 +4424,7 @@
         <v>154</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C155" s="1" t="s">
         <v>14</v>
@@ -4439,7 +4439,7 @@
         <v>4</v>
       </c>
       <c r="G155" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="156" spans="1:7" x14ac:dyDescent="0.2">
@@ -4447,13 +4447,13 @@
         <v>155</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C156" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E156" s="2">
         <v>5908071</v>
@@ -4462,7 +4462,7 @@
         <v>4</v>
       </c>
       <c r="G156" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="157" spans="1:7" x14ac:dyDescent="0.2">
@@ -4470,13 +4470,13 @@
         <v>156</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C157" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E157" s="2">
         <v>179101</v>
@@ -4485,7 +4485,7 @@
         <v>4</v>
       </c>
       <c r="G157" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="158" spans="1:7" x14ac:dyDescent="0.2">
@@ -4493,13 +4493,13 @@
         <v>157</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C158" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E158" s="2">
         <v>257494</v>
@@ -4508,7 +4508,7 @@
         <v>4</v>
       </c>
       <c r="G158" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="159" spans="1:7" x14ac:dyDescent="0.2">
@@ -4516,13 +4516,13 @@
         <v>158</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C159" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E159" s="2">
         <v>3078049</v>
@@ -4531,7 +4531,7 @@
         <v>4</v>
       </c>
       <c r="G159" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="160" spans="1:7" x14ac:dyDescent="0.2">
@@ -4539,7 +4539,7 @@
         <v>159</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C160" s="1" t="s">
         <v>14</v>
@@ -4554,7 +4554,7 @@
         <v>4</v>
       </c>
       <c r="G160" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="161" spans="1:7" x14ac:dyDescent="0.2">
@@ -4562,7 +4562,7 @@
         <v>160</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C161" s="1" t="s">
         <v>14</v>
@@ -4577,7 +4577,7 @@
         <v>4</v>
       </c>
       <c r="G161" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="162" spans="1:7" x14ac:dyDescent="0.2">
@@ -4585,13 +4585,13 @@
         <v>161</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C162" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D162" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E162" s="2">
         <v>54520</v>
@@ -4600,7 +4600,7 @@
         <v>4</v>
       </c>
       <c r="G162" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="163" spans="1:7" x14ac:dyDescent="0.2">
@@ -4608,7 +4608,7 @@
         <v>162</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C163" s="1" t="s">
         <v>35</v>
@@ -4620,10 +4620,10 @@
         <v>3807115500</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G163" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="164" spans="1:7" x14ac:dyDescent="0.2">
@@ -4631,22 +4631,22 @@
         <v>163</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C164" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E164" s="2">
         <v>1950000</v>
       </c>
       <c r="F164" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G164" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="165" spans="1:7" x14ac:dyDescent="0.2">
@@ -4654,22 +4654,22 @@
         <v>164</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C165" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D165" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E165" s="2">
         <v>1600000</v>
       </c>
       <c r="F165" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G165" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="166" spans="1:7" x14ac:dyDescent="0.2">
@@ -4677,22 +4677,22 @@
         <v>165</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C166" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D166" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E166" s="2">
         <v>90000000</v>
       </c>
       <c r="F166" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G166" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="167" spans="1:7" x14ac:dyDescent="0.2">
@@ -4700,22 +4700,22 @@
         <v>166</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C167" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D167" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E167" s="2">
         <v>637700000</v>
       </c>
       <c r="F167" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G167" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="168" spans="1:7" x14ac:dyDescent="0.2">
@@ -4723,22 +4723,22 @@
         <v>167</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C168" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D168" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E168" s="2">
         <v>1273100000</v>
       </c>
       <c r="F168" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G168" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="169" spans="1:7" x14ac:dyDescent="0.2">
@@ -4746,22 +4746,22 @@
         <v>168</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C169" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D169" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E169" s="2">
         <v>174420000</v>
       </c>
       <c r="F169" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G169" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="170" spans="1:7" x14ac:dyDescent="0.2">
@@ -4769,22 +4769,22 @@
         <v>169</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C170" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D170" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E170" s="2">
         <v>1000000</v>
       </c>
       <c r="F170" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G170" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="171" spans="1:7" x14ac:dyDescent="0.2">
@@ -4792,7 +4792,7 @@
         <v>170</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>14</v>
@@ -4804,10 +4804,10 @@
         <v>147000000</v>
       </c>
       <c r="F171" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G171" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="172" spans="1:7" x14ac:dyDescent="0.2">
@@ -4815,7 +4815,7 @@
         <v>171</v>
       </c>
       <c r="B172" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C172" s="1" t="s">
         <v>14</v>
@@ -4827,10 +4827,10 @@
         <v>40000000</v>
       </c>
       <c r="F172" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G172" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="173" spans="1:7" x14ac:dyDescent="0.2">
@@ -4838,7 +4838,7 @@
         <v>172</v>
       </c>
       <c r="B173" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C173" s="1" t="s">
         <v>14</v>
@@ -4850,10 +4850,10 @@
         <v>1000000</v>
       </c>
       <c r="F173" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G173" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="174" spans="1:7" x14ac:dyDescent="0.2">
@@ -4861,22 +4861,22 @@
         <v>173</v>
       </c>
       <c r="B174" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C174" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D174" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E174" s="2">
         <v>21220000</v>
       </c>
       <c r="F174" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G174" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="175" spans="1:7" x14ac:dyDescent="0.2">
@@ -4884,7 +4884,7 @@
         <v>174</v>
       </c>
       <c r="B175" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C175" s="1" t="s">
         <v>14</v>
@@ -4896,10 +4896,10 @@
         <v>28300000</v>
       </c>
       <c r="F175" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G175" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="176" spans="1:7" x14ac:dyDescent="0.2">
@@ -4907,22 +4907,22 @@
         <v>175</v>
       </c>
       <c r="B176" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C176" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D176" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E176" s="2">
         <v>15700500</v>
       </c>
       <c r="F176" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G176" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="177" spans="1:7" x14ac:dyDescent="0.2">
@@ -4930,22 +4930,22 @@
         <v>176</v>
       </c>
       <c r="B177" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C177" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D177" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E177" s="2">
         <v>6000000</v>
       </c>
       <c r="F177" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G177" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="178" spans="1:7" x14ac:dyDescent="0.2">
@@ -4953,22 +4953,22 @@
         <v>177</v>
       </c>
       <c r="B178" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C178" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D178" s="1" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E178" s="2">
         <v>125100000</v>
       </c>
       <c r="F178" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G178" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="179" spans="1:7" x14ac:dyDescent="0.2">
@@ -4976,22 +4976,22 @@
         <v>178</v>
       </c>
       <c r="B179" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C179" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D179" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E179" s="2">
         <v>6825000</v>
       </c>
       <c r="F179" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G179" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="180" spans="1:7" x14ac:dyDescent="0.2">
@@ -4999,7 +4999,7 @@
         <v>179</v>
       </c>
       <c r="B180" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C180" s="1" t="s">
         <v>14</v>
@@ -5011,10 +5011,10 @@
         <v>179400000</v>
       </c>
       <c r="F180" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G180" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="181" spans="1:7" x14ac:dyDescent="0.2">
@@ -5022,7 +5022,7 @@
         <v>180</v>
       </c>
       <c r="B181" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C181" s="1" t="s">
         <v>14</v>
@@ -5034,10 +5034,10 @@
         <v>1045500000</v>
       </c>
       <c r="F181" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G181" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="182" spans="1:7" x14ac:dyDescent="0.2">
@@ -5045,22 +5045,22 @@
         <v>181</v>
       </c>
       <c r="B182" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C182" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D182" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E182" s="2">
         <v>11300000</v>
       </c>
       <c r="F182" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="G182" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="183" spans="1:7" x14ac:dyDescent="0.2">
@@ -5068,7 +5068,7 @@
         <v>182</v>
       </c>
       <c r="B183" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C183" s="1" t="s">
         <v>35</v>
@@ -5083,7 +5083,7 @@
         <v>58</v>
       </c>
       <c r="G183" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="184" spans="1:7" x14ac:dyDescent="0.2">
@@ -5091,13 +5091,13 @@
         <v>183</v>
       </c>
       <c r="B184" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C184" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D184" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E184" s="2">
         <v>164318</v>
@@ -5106,7 +5106,7 @@
         <v>58</v>
       </c>
       <c r="G184" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="185" spans="1:7" x14ac:dyDescent="0.2">
@@ -5114,13 +5114,13 @@
         <v>184</v>
       </c>
       <c r="B185" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C185" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D185" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E185" s="2">
         <v>788805</v>
@@ -5129,7 +5129,7 @@
         <v>58</v>
       </c>
       <c r="G185" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="186" spans="1:7" x14ac:dyDescent="0.2">
@@ -5137,13 +5137,13 @@
         <v>185</v>
       </c>
       <c r="B186" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C186" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D186" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E186" s="2">
         <v>3403830</v>
@@ -5152,7 +5152,7 @@
         <v>58</v>
       </c>
       <c r="G186" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.2">
@@ -5160,13 +5160,13 @@
         <v>190</v>
       </c>
       <c r="B187" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C187" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D187" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E187" s="2">
         <v>4779094</v>
@@ -5175,7 +5175,7 @@
         <v>58</v>
       </c>
       <c r="G187" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="188" spans="1:7" x14ac:dyDescent="0.2">
@@ -5183,13 +5183,13 @@
         <v>191</v>
       </c>
       <c r="B188" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C188" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D188" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E188" s="2">
         <v>1999377</v>
@@ -5198,7 +5198,7 @@
         <v>58</v>
       </c>
       <c r="G188" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.2">
@@ -5206,13 +5206,13 @@
         <v>192</v>
       </c>
       <c r="B189" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C189" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D189" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E189" s="2">
         <v>4218107</v>
@@ -5221,7 +5221,7 @@
         <v>58</v>
       </c>
       <c r="G189" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.2">
@@ -5229,7 +5229,7 @@
         <v>193</v>
       </c>
       <c r="B190" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C190" s="1" t="s">
         <v>14</v>
@@ -5244,7 +5244,7 @@
         <v>58</v>
       </c>
       <c r="G190" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.2">
@@ -5252,7 +5252,7 @@
         <v>197</v>
       </c>
       <c r="B191" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C191" s="1" t="s">
         <v>14</v>
@@ -5267,7 +5267,7 @@
         <v>58</v>
       </c>
       <c r="G191" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.2">
@@ -5275,7 +5275,7 @@
         <v>198</v>
       </c>
       <c r="B192" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C192" s="1" t="s">
         <v>14</v>
@@ -5290,7 +5290,7 @@
         <v>58</v>
       </c>
       <c r="G192" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.2">
@@ -5298,7 +5298,7 @@
         <v>199</v>
       </c>
       <c r="B193" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C193" s="1" t="s">
         <v>14</v>
@@ -5313,7 +5313,7 @@
         <v>58</v>
       </c>
       <c r="G193" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="194" spans="1:7" x14ac:dyDescent="0.2">
@@ -5321,13 +5321,13 @@
         <v>200</v>
       </c>
       <c r="B194" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C194" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D194" s="1" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E194" s="2">
         <v>11959114</v>
@@ -5336,7 +5336,7 @@
         <v>58</v>
       </c>
       <c r="G194" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.2">
@@ -5344,7 +5344,7 @@
         <v>204</v>
       </c>
       <c r="B195" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C195" s="1" t="s">
         <v>14</v>
@@ -5359,7 +5359,7 @@
         <v>58</v>
       </c>
       <c r="G195" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="196" spans="1:7" x14ac:dyDescent="0.2">
@@ -5367,13 +5367,13 @@
         <v>205</v>
       </c>
       <c r="B196" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C196" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D196" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E196" s="2">
         <v>2767341</v>
@@ -5382,7 +5382,7 @@
         <v>58</v>
       </c>
       <c r="G196" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="197" spans="1:7" x14ac:dyDescent="0.2">
@@ -5390,13 +5390,13 @@
         <v>206</v>
       </c>
       <c r="B197" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C197" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D197" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E197" s="2">
         <v>297864</v>
@@ -5405,7 +5405,7 @@
         <v>58</v>
       </c>
       <c r="G197" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="198" spans="1:7" x14ac:dyDescent="0.2">
@@ -5413,13 +5413,13 @@
         <v>207</v>
       </c>
       <c r="B198" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C198" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D198" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E198" s="2">
         <v>373282</v>
@@ -5428,7 +5428,7 @@
         <v>58</v>
       </c>
       <c r="G198" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="199" spans="1:7" x14ac:dyDescent="0.2">
@@ -5436,13 +5436,13 @@
         <v>208</v>
       </c>
       <c r="B199" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C199" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D199" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E199" s="2">
         <v>979534</v>
@@ -5451,7 +5451,7 @@
         <v>58</v>
       </c>
       <c r="G199" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.2">
@@ -5459,7 +5459,7 @@
         <v>212</v>
       </c>
       <c r="B200" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C200" s="1" t="s">
         <v>14</v>
@@ -5474,7 +5474,7 @@
         <v>58</v>
       </c>
       <c r="G200" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.2">
@@ -5482,7 +5482,7 @@
         <v>213</v>
       </c>
       <c r="B201" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C201" s="1" t="s">
         <v>14</v>
@@ -5497,7 +5497,7 @@
         <v>58</v>
       </c>
       <c r="G201" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="202" spans="1:7" x14ac:dyDescent="0.2">
@@ -5505,13 +5505,13 @@
         <v>214</v>
       </c>
       <c r="B202" s="1" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C202" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D202" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E202" s="2">
         <v>1916809</v>
@@ -5520,7 +5520,7 @@
         <v>58</v>
       </c>
       <c r="G202" s="1" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="203" spans="1:7" x14ac:dyDescent="0.2">
@@ -5528,13 +5528,13 @@
         <v>222</v>
       </c>
       <c r="B203" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C203" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D203" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E203" s="2">
         <v>247300</v>
@@ -5543,7 +5543,7 @@
         <v>74</v>
       </c>
       <c r="G203" s="1" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="204" spans="1:7" x14ac:dyDescent="0.2">
@@ -5551,13 +5551,13 @@
         <v>223</v>
       </c>
       <c r="B204" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C204" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D204" s="1" t="s">
         <v>130</v>
-      </c>
-      <c r="C204" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D204" s="1" t="s">
-        <v>131</v>
       </c>
       <c r="E204" s="2">
         <v>415110</v>
@@ -5566,7 +5566,7 @@
         <v>74</v>
       </c>
       <c r="G204" s="1" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.2">
@@ -5574,13 +5574,13 @@
         <v>224</v>
       </c>
       <c r="B205" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C205" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D205" s="1" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E205" s="2">
         <v>1054400</v>
@@ -5589,7 +5589,7 @@
         <v>74</v>
       </c>
       <c r="G205" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.2">
@@ -5597,13 +5597,13 @@
         <v>225</v>
       </c>
       <c r="B206" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C206" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D206" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E206" s="2">
         <v>535275</v>
@@ -5612,7 +5612,7 @@
         <v>74</v>
       </c>
       <c r="G206" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
     </row>
     <row r="207" spans="1:7" x14ac:dyDescent="0.2">
@@ -5620,13 +5620,13 @@
         <v>226</v>
       </c>
       <c r="B207" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C207" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D207" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E207" s="2">
         <v>4917340</v>
@@ -5635,7 +5635,7 @@
         <v>74</v>
       </c>
       <c r="G207" s="1" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="208" spans="1:7" x14ac:dyDescent="0.2">
@@ -5643,13 +5643,13 @@
         <v>227</v>
       </c>
       <c r="B208" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C208" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D208" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E208" s="2">
         <v>322930</v>
@@ -5658,7 +5658,7 @@
         <v>74</v>
       </c>
       <c r="G208" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.2">
@@ -5666,7 +5666,7 @@
         <v>228</v>
       </c>
       <c r="B209" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C209" s="1" t="s">
         <v>14</v>
@@ -5681,7 +5681,7 @@
         <v>74</v>
       </c>
       <c r="G209" s="1" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.2">
@@ -5689,7 +5689,7 @@
         <v>229</v>
       </c>
       <c r="B210" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C210" s="1" t="s">
         <v>14</v>
@@ -5704,7 +5704,7 @@
         <v>74</v>
       </c>
       <c r="G210" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.2">
@@ -5712,13 +5712,13 @@
         <v>230</v>
       </c>
       <c r="B211" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C211" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D211" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E211" s="2">
         <v>1930412</v>
@@ -5735,7 +5735,7 @@
         <v>231</v>
       </c>
       <c r="B212" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C212" s="1" t="s">
         <v>14</v>
@@ -5750,7 +5750,7 @@
         <v>74</v>
       </c>
       <c r="G212" s="1" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.2">
@@ -5758,13 +5758,13 @@
         <v>232</v>
       </c>
       <c r="B213" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C213" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D213" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E213" s="2">
         <v>520360</v>
@@ -5773,7 +5773,7 @@
         <v>74</v>
       </c>
       <c r="G213" s="1" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.2">
@@ -5781,13 +5781,13 @@
         <v>233</v>
       </c>
       <c r="B214" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C214" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D214" s="1" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E214" s="2">
         <v>436420</v>
@@ -5796,7 +5796,7 @@
         <v>74</v>
       </c>
       <c r="G214" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.2">
@@ -5804,13 +5804,13 @@
         <v>234</v>
       </c>
       <c r="B215" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C215" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D215" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E215" s="2">
         <v>255950</v>
@@ -5819,7 +5819,7 @@
         <v>74</v>
       </c>
       <c r="G215" s="1" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.2">
@@ -5827,13 +5827,13 @@
         <v>235</v>
       </c>
       <c r="B216" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C216" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D216" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E216" s="2">
         <v>36440</v>
@@ -5850,13 +5850,13 @@
         <v>236</v>
       </c>
       <c r="B217" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C217" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D217" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E217" s="2">
         <v>673560</v>
@@ -5873,13 +5873,13 @@
         <v>237</v>
       </c>
       <c r="B218" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C218" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D218" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E218" s="2">
         <v>462055</v>
@@ -5888,7 +5888,7 @@
         <v>74</v>
       </c>
       <c r="G218" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.2">
@@ -5896,7 +5896,7 @@
         <v>238</v>
       </c>
       <c r="B219" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C219" s="1" t="s">
         <v>14</v>
@@ -5911,7 +5911,7 @@
         <v>74</v>
       </c>
       <c r="G219" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.2">
@@ -5919,7 +5919,7 @@
         <v>239</v>
       </c>
       <c r="B220" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C220" s="1" t="s">
         <v>14</v>
@@ -5934,7 +5934,7 @@
         <v>74</v>
       </c>
       <c r="G220" s="1" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.2">
@@ -5942,13 +5942,13 @@
         <v>240</v>
       </c>
       <c r="B221" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C221" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D221" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E221" s="2">
         <v>177310</v>
@@ -5957,7 +5957,7 @@
         <v>74</v>
       </c>
       <c r="G221" s="1" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.2">
@@ -5965,7 +5965,7 @@
         <v>241</v>
       </c>
       <c r="B222" s="1" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C222" s="1" t="s">
         <v>35</v>
@@ -5980,7 +5980,7 @@
         <v>74</v>
       </c>
       <c r="G222" s="1" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.2">
@@ -5988,22 +5988,22 @@
         <v>242</v>
       </c>
       <c r="B223" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C223" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D223" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E223" s="2">
         <v>2346091355</v>
       </c>
       <c r="F223" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G223" s="1" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.2">
@@ -6011,22 +6011,22 @@
         <v>243</v>
       </c>
       <c r="B224" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C224" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D224" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E224" s="2">
         <v>2053518805</v>
       </c>
       <c r="F224" t="s">
+        <v>153</v>
+      </c>
+      <c r="G224" s="1" t="s">
         <v>154</v>
-      </c>
-      <c r="G224" s="1" t="s">
-        <v>155</v>
       </c>
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.2">
@@ -6034,22 +6034,22 @@
         <v>244</v>
       </c>
       <c r="B225" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C225" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D225" s="1" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="E225" s="2">
         <v>27255662244</v>
       </c>
       <c r="F225" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G225" s="1" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.2">
@@ -6057,22 +6057,22 @@
         <v>245</v>
       </c>
       <c r="B226" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C226" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D226" s="1" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E226" s="2">
         <v>5195094477</v>
       </c>
       <c r="F226" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G226" s="1" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.2">
@@ -6080,22 +6080,22 @@
         <v>246</v>
       </c>
       <c r="B227" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C227" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D227" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E227" s="2">
         <v>10244621028</v>
       </c>
       <c r="F227" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G227" s="1" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.2">
@@ -6103,22 +6103,22 @@
         <v>247</v>
       </c>
       <c r="B228" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C228" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D228" s="1" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E228" s="2">
         <v>2225685962</v>
       </c>
       <c r="F228" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G228" s="1" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.2">
@@ -6126,7 +6126,7 @@
         <v>248</v>
       </c>
       <c r="B229" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C229" s="1" t="s">
         <v>14</v>
@@ -6138,7 +6138,7 @@
         <v>8887960226</v>
       </c>
       <c r="F229" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G229" s="1" t="s">
         <v>75</v>
@@ -6149,7 +6149,7 @@
         <v>249</v>
       </c>
       <c r="B230" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C230" s="1" t="s">
         <v>14</v>
@@ -6161,10 +6161,10 @@
         <v>13484064490</v>
       </c>
       <c r="F230" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G230" s="1" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.2">
@@ -6172,7 +6172,7 @@
         <v>250</v>
       </c>
       <c r="B231" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C231" s="1" t="s">
         <v>14</v>
@@ -6184,7 +6184,7 @@
         <v>28723043437</v>
       </c>
       <c r="F231" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G231" s="1" t="s">
         <v>59</v>
@@ -6195,7 +6195,7 @@
         <v>251</v>
       </c>
       <c r="B232" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C232" s="1" t="s">
         <v>14</v>
@@ -6207,7 +6207,7 @@
         <v>7281805328</v>
       </c>
       <c r="F232" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G232" s="1" t="s">
         <v>63</v>
@@ -6218,19 +6218,19 @@
         <v>252</v>
       </c>
       <c r="B233" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C233" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D233" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E233" s="2">
         <v>1464725845</v>
       </c>
       <c r="F233" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G233" s="1" t="s">
         <v>66</v>
@@ -6241,7 +6241,7 @@
         <v>253</v>
       </c>
       <c r="B234" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C234" s="1" t="s">
         <v>14</v>
@@ -6253,10 +6253,10 @@
         <v>1950922906</v>
       </c>
       <c r="F234" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G234" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.2">
@@ -6264,19 +6264,19 @@
         <v>254</v>
       </c>
       <c r="B235" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C235" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D235" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E235" s="2">
         <v>885932730</v>
       </c>
       <c r="F235" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G235" s="1" t="s">
         <v>70</v>
@@ -6287,22 +6287,22 @@
         <v>255</v>
       </c>
       <c r="B236" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C236" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D236" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E236" s="2">
         <v>11068089527</v>
       </c>
       <c r="F236" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G236" s="1" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.2">
@@ -6310,22 +6310,22 @@
         <v>256</v>
       </c>
       <c r="B237" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C237" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D237" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E237" s="2">
         <v>14671014464</v>
       </c>
       <c r="F237" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G237" s="1" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.2">
@@ -6333,22 +6333,22 @@
         <v>257</v>
       </c>
       <c r="B238" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C238" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D238" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E238" s="2">
         <v>10589643004</v>
       </c>
       <c r="F238" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G238" s="1" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.2">
@@ -6356,7 +6356,7 @@
         <v>258</v>
       </c>
       <c r="B239" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C239" s="1" t="s">
         <v>14</v>
@@ -6368,10 +6368,10 @@
         <v>3252244500</v>
       </c>
       <c r="F239" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G239" s="1" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.2">
@@ -6379,7 +6379,7 @@
         <v>259</v>
       </c>
       <c r="B240" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C240" s="1" t="s">
         <v>14</v>
@@ -6391,10 +6391,10 @@
         <v>4191108684</v>
       </c>
       <c r="F240" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G240" s="1" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
     </row>
     <row r="241" spans="1:7" x14ac:dyDescent="0.2">
@@ -6402,19 +6402,19 @@
         <v>260</v>
       </c>
       <c r="B241" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C241" s="1" t="s">
         <v>14</v>
       </c>
       <c r="D241" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E241" s="2">
         <v>4937711997</v>
       </c>
       <c r="F241" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G241" s="1" t="s">
         <v>86</v>
@@ -6425,7 +6425,7 @@
         <v>261</v>
       </c>
       <c r="B242" s="1" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C242" s="1" t="s">
         <v>35</v>
@@ -6437,10 +6437,10 @@
         <v>160708941019</v>
       </c>
       <c r="F242" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="G242" s="1" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
still a work in progress, finalizing data entry
</commit_message>
<xml_diff>
--- a/data/raw/raw summary cost data.xlsx
+++ b/data/raw/raw summary cost data.xlsx
@@ -8,19 +8,31 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/stepheaneff/Documents/work/GT/costed-NAPHS/data/raw/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{86DA06D1-6527-C441-8E30-B0ED37A11119}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BA0BD89F-6F21-0E4E-AC02-AE7B4525E19C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3660" yWindow="760" windowWidth="26580" windowHeight="13180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="181029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1212" uniqueCount="167">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="186">
   <si>
     <t>country</t>
   </si>
@@ -521,13 +533,70 @@
   </si>
   <si>
     <t>Zoonotic events and the human-animal interface</t>
+  </si>
+  <si>
+    <t>North Macedonia</t>
+  </si>
+  <si>
+    <t>Legislation and Financing</t>
+  </si>
+  <si>
+    <t>USD (2023)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Zoonotic Disease </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Food Safety </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Biosafety and Biosecurity </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Immunization </t>
+  </si>
+  <si>
+    <t xml:space="preserve">National Laboratory System </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Real-Time Surveillance </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Reporting </t>
+  </si>
+  <si>
+    <t>Human Resoures (Animal and human health sector)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preparedness </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Emergency Response Operations </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linking Public Health and Security Authorities </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Medical Countermeasures </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Risk Communication </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Events Points of Entry (PoEs) </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Chemical Events </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Radiation Emergencies </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -540,6 +609,19 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -562,20 +644,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="3" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -880,11 +965,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G242"/>
+  <dimension ref="A1:G262"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.33203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="10.5" style="1" customWidth="1"/>
+    <col min="2" max="2" width="19.5" style="1" customWidth="1"/>
     <col min="3" max="3" width="21" style="1" customWidth="1"/>
     <col min="4" max="4" width="23.6640625" style="1" customWidth="1"/>
     <col min="5" max="6" width="16.83203125" style="1" customWidth="1"/>
@@ -5157,7 +5242,7 @@
     </row>
     <row r="187" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A187" s="1">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B187" s="1" t="s">
         <v>127</v>
@@ -5180,7 +5265,7 @@
     </row>
     <row r="188" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A188" s="1">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B188" s="1" t="s">
         <v>127</v>
@@ -5203,7 +5288,7 @@
     </row>
     <row r="189" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A189" s="1">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B189" s="1" t="s">
         <v>127</v>
@@ -5226,7 +5311,7 @@
     </row>
     <row r="190" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A190" s="1">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B190" s="1" t="s">
         <v>127</v>
@@ -5249,7 +5334,7 @@
     </row>
     <row r="191" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A191" s="1">
-        <v>197</v>
+        <v>190</v>
       </c>
       <c r="B191" s="1" t="s">
         <v>127</v>
@@ -5272,7 +5357,7 @@
     </row>
     <row r="192" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A192" s="1">
-        <v>198</v>
+        <v>191</v>
       </c>
       <c r="B192" s="1" t="s">
         <v>127</v>
@@ -5295,7 +5380,7 @@
     </row>
     <row r="193" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A193" s="1">
-        <v>199</v>
+        <v>192</v>
       </c>
       <c r="B193" s="1" t="s">
         <v>127</v>
@@ -5318,7 +5403,7 @@
     </row>
     <row r="194" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A194" s="1">
-        <v>200</v>
+        <v>193</v>
       </c>
       <c r="B194" s="1" t="s">
         <v>127</v>
@@ -5341,7 +5426,7 @@
     </row>
     <row r="195" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A195" s="1">
-        <v>204</v>
+        <v>194</v>
       </c>
       <c r="B195" s="1" t="s">
         <v>127</v>
@@ -5364,7 +5449,7 @@
     </row>
     <row r="196" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A196" s="1">
-        <v>205</v>
+        <v>195</v>
       </c>
       <c r="B196" s="1" t="s">
         <v>127</v>
@@ -5387,7 +5472,7 @@
     </row>
     <row r="197" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A197" s="1">
-        <v>206</v>
+        <v>196</v>
       </c>
       <c r="B197" s="1" t="s">
         <v>127</v>
@@ -5410,7 +5495,7 @@
     </row>
     <row r="198" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A198" s="1">
-        <v>207</v>
+        <v>197</v>
       </c>
       <c r="B198" s="1" t="s">
         <v>127</v>
@@ -5433,7 +5518,7 @@
     </row>
     <row r="199" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A199" s="1">
-        <v>208</v>
+        <v>198</v>
       </c>
       <c r="B199" s="1" t="s">
         <v>127</v>
@@ -5456,7 +5541,7 @@
     </row>
     <row r="200" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A200" s="1">
-        <v>212</v>
+        <v>199</v>
       </c>
       <c r="B200" s="1" t="s">
         <v>127</v>
@@ -5479,7 +5564,7 @@
     </row>
     <row r="201" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A201" s="1">
-        <v>213</v>
+        <v>200</v>
       </c>
       <c r="B201" s="1" t="s">
         <v>127</v>
@@ -5502,7 +5587,7 @@
     </row>
     <row r="202" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A202" s="1">
-        <v>214</v>
+        <v>201</v>
       </c>
       <c r="B202" s="1" t="s">
         <v>127</v>
@@ -5525,7 +5610,7 @@
     </row>
     <row r="203" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A203" s="1">
-        <v>222</v>
+        <v>202</v>
       </c>
       <c r="B203" s="1" t="s">
         <v>129</v>
@@ -5548,7 +5633,7 @@
     </row>
     <row r="204" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A204" s="1">
-        <v>223</v>
+        <v>203</v>
       </c>
       <c r="B204" s="1" t="s">
         <v>129</v>
@@ -5571,7 +5656,7 @@
     </row>
     <row r="205" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A205" s="1">
-        <v>224</v>
+        <v>204</v>
       </c>
       <c r="B205" s="1" t="s">
         <v>129</v>
@@ -5594,7 +5679,7 @@
     </row>
     <row r="206" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A206" s="1">
-        <v>225</v>
+        <v>205</v>
       </c>
       <c r="B206" s="1" t="s">
         <v>129</v>
@@ -5617,7 +5702,7 @@
     </row>
     <row r="207" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A207" s="1">
-        <v>226</v>
+        <v>206</v>
       </c>
       <c r="B207" s="1" t="s">
         <v>129</v>
@@ -5640,7 +5725,7 @@
     </row>
     <row r="208" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A208" s="1">
-        <v>227</v>
+        <v>207</v>
       </c>
       <c r="B208" s="1" t="s">
         <v>129</v>
@@ -5663,7 +5748,7 @@
     </row>
     <row r="209" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A209" s="1">
-        <v>228</v>
+        <v>208</v>
       </c>
       <c r="B209" s="1" t="s">
         <v>129</v>
@@ -5686,7 +5771,7 @@
     </row>
     <row r="210" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A210" s="1">
-        <v>229</v>
+        <v>209</v>
       </c>
       <c r="B210" s="1" t="s">
         <v>129</v>
@@ -5709,7 +5794,7 @@
     </row>
     <row r="211" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A211" s="1">
-        <v>230</v>
+        <v>210</v>
       </c>
       <c r="B211" s="1" t="s">
         <v>129</v>
@@ -5732,7 +5817,7 @@
     </row>
     <row r="212" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A212" s="1">
-        <v>231</v>
+        <v>211</v>
       </c>
       <c r="B212" s="1" t="s">
         <v>129</v>
@@ -5755,7 +5840,7 @@
     </row>
     <row r="213" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A213" s="1">
-        <v>232</v>
+        <v>212</v>
       </c>
       <c r="B213" s="1" t="s">
         <v>129</v>
@@ -5778,7 +5863,7 @@
     </row>
     <row r="214" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A214" s="1">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="B214" s="1" t="s">
         <v>129</v>
@@ -5801,7 +5886,7 @@
     </row>
     <row r="215" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A215" s="1">
-        <v>234</v>
+        <v>214</v>
       </c>
       <c r="B215" s="1" t="s">
         <v>129</v>
@@ -5824,7 +5909,7 @@
     </row>
     <row r="216" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A216" s="1">
-        <v>235</v>
+        <v>215</v>
       </c>
       <c r="B216" s="1" t="s">
         <v>129</v>
@@ -5847,7 +5932,7 @@
     </row>
     <row r="217" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A217" s="1">
-        <v>236</v>
+        <v>216</v>
       </c>
       <c r="B217" s="1" t="s">
         <v>129</v>
@@ -5870,7 +5955,7 @@
     </row>
     <row r="218" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A218" s="1">
-        <v>237</v>
+        <v>217</v>
       </c>
       <c r="B218" s="1" t="s">
         <v>129</v>
@@ -5893,7 +5978,7 @@
     </row>
     <row r="219" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A219" s="1">
-        <v>238</v>
+        <v>218</v>
       </c>
       <c r="B219" s="1" t="s">
         <v>129</v>
@@ -5916,7 +6001,7 @@
     </row>
     <row r="220" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A220" s="1">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="B220" s="1" t="s">
         <v>129</v>
@@ -5939,7 +6024,7 @@
     </row>
     <row r="221" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A221" s="1">
-        <v>240</v>
+        <v>220</v>
       </c>
       <c r="B221" s="1" t="s">
         <v>129</v>
@@ -5962,7 +6047,7 @@
     </row>
     <row r="222" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A222" s="1">
-        <v>241</v>
+        <v>221</v>
       </c>
       <c r="B222" s="1" t="s">
         <v>129</v>
@@ -5985,7 +6070,7 @@
     </row>
     <row r="223" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A223" s="1">
-        <v>242</v>
+        <v>222</v>
       </c>
       <c r="B223" s="1" t="s">
         <v>150</v>
@@ -5999,7 +6084,7 @@
       <c r="E223" s="2">
         <v>2346091355</v>
       </c>
-      <c r="F223" t="s">
+      <c r="F223" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G223" s="1" t="s">
@@ -6008,7 +6093,7 @@
     </row>
     <row r="224" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A224" s="1">
-        <v>243</v>
+        <v>223</v>
       </c>
       <c r="B224" s="1" t="s">
         <v>150</v>
@@ -6022,7 +6107,7 @@
       <c r="E224" s="2">
         <v>2053518805</v>
       </c>
-      <c r="F224" t="s">
+      <c r="F224" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G224" s="1" t="s">
@@ -6031,7 +6116,7 @@
     </row>
     <row r="225" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A225" s="1">
-        <v>244</v>
+        <v>224</v>
       </c>
       <c r="B225" s="1" t="s">
         <v>150</v>
@@ -6045,7 +6130,7 @@
       <c r="E225" s="2">
         <v>27255662244</v>
       </c>
-      <c r="F225" t="s">
+      <c r="F225" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G225" s="1" t="s">
@@ -6054,7 +6139,7 @@
     </row>
     <row r="226" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A226" s="1">
-        <v>245</v>
+        <v>225</v>
       </c>
       <c r="B226" s="1" t="s">
         <v>150</v>
@@ -6068,7 +6153,7 @@
       <c r="E226" s="2">
         <v>5195094477</v>
       </c>
-      <c r="F226" t="s">
+      <c r="F226" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G226" s="1" t="s">
@@ -6077,7 +6162,7 @@
     </row>
     <row r="227" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A227" s="1">
-        <v>246</v>
+        <v>226</v>
       </c>
       <c r="B227" s="1" t="s">
         <v>150</v>
@@ -6091,7 +6176,7 @@
       <c r="E227" s="2">
         <v>10244621028</v>
       </c>
-      <c r="F227" t="s">
+      <c r="F227" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G227" s="1" t="s">
@@ -6100,7 +6185,7 @@
     </row>
     <row r="228" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A228" s="1">
-        <v>247</v>
+        <v>227</v>
       </c>
       <c r="B228" s="1" t="s">
         <v>150</v>
@@ -6114,7 +6199,7 @@
       <c r="E228" s="2">
         <v>2225685962</v>
       </c>
-      <c r="F228" t="s">
+      <c r="F228" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G228" s="1" t="s">
@@ -6123,7 +6208,7 @@
     </row>
     <row r="229" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A229" s="1">
-        <v>248</v>
+        <v>228</v>
       </c>
       <c r="B229" s="1" t="s">
         <v>150</v>
@@ -6137,7 +6222,7 @@
       <c r="E229" s="2">
         <v>8887960226</v>
       </c>
-      <c r="F229" t="s">
+      <c r="F229" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G229" s="1" t="s">
@@ -6146,7 +6231,7 @@
     </row>
     <row r="230" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A230" s="1">
-        <v>249</v>
+        <v>229</v>
       </c>
       <c r="B230" s="1" t="s">
         <v>150</v>
@@ -6160,7 +6245,7 @@
       <c r="E230" s="2">
         <v>13484064490</v>
       </c>
-      <c r="F230" t="s">
+      <c r="F230" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G230" s="1" t="s">
@@ -6169,7 +6254,7 @@
     </row>
     <row r="231" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A231" s="1">
-        <v>250</v>
+        <v>230</v>
       </c>
       <c r="B231" s="1" t="s">
         <v>150</v>
@@ -6183,7 +6268,7 @@
       <c r="E231" s="2">
         <v>28723043437</v>
       </c>
-      <c r="F231" t="s">
+      <c r="F231" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G231" s="1" t="s">
@@ -6192,7 +6277,7 @@
     </row>
     <row r="232" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A232" s="1">
-        <v>251</v>
+        <v>231</v>
       </c>
       <c r="B232" s="1" t="s">
         <v>150</v>
@@ -6206,7 +6291,7 @@
       <c r="E232" s="2">
         <v>7281805328</v>
       </c>
-      <c r="F232" t="s">
+      <c r="F232" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G232" s="1" t="s">
@@ -6215,7 +6300,7 @@
     </row>
     <row r="233" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A233" s="1">
-        <v>252</v>
+        <v>232</v>
       </c>
       <c r="B233" s="1" t="s">
         <v>150</v>
@@ -6229,7 +6314,7 @@
       <c r="E233" s="2">
         <v>1464725845</v>
       </c>
-      <c r="F233" t="s">
+      <c r="F233" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G233" s="1" t="s">
@@ -6238,7 +6323,7 @@
     </row>
     <row r="234" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A234" s="1">
-        <v>253</v>
+        <v>233</v>
       </c>
       <c r="B234" s="1" t="s">
         <v>150</v>
@@ -6252,7 +6337,7 @@
       <c r="E234" s="2">
         <v>1950922906</v>
       </c>
-      <c r="F234" t="s">
+      <c r="F234" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G234" s="1" t="s">
@@ -6261,7 +6346,7 @@
     </row>
     <row r="235" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A235" s="1">
-        <v>254</v>
+        <v>234</v>
       </c>
       <c r="B235" s="1" t="s">
         <v>150</v>
@@ -6275,7 +6360,7 @@
       <c r="E235" s="2">
         <v>885932730</v>
       </c>
-      <c r="F235" t="s">
+      <c r="F235" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G235" s="1" t="s">
@@ -6284,7 +6369,7 @@
     </row>
     <row r="236" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A236" s="1">
-        <v>255</v>
+        <v>235</v>
       </c>
       <c r="B236" s="1" t="s">
         <v>150</v>
@@ -6298,7 +6383,7 @@
       <c r="E236" s="2">
         <v>11068089527</v>
       </c>
-      <c r="F236" t="s">
+      <c r="F236" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G236" s="1" t="s">
@@ -6307,7 +6392,7 @@
     </row>
     <row r="237" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A237" s="1">
-        <v>256</v>
+        <v>236</v>
       </c>
       <c r="B237" s="1" t="s">
         <v>150</v>
@@ -6321,7 +6406,7 @@
       <c r="E237" s="2">
         <v>14671014464</v>
       </c>
-      <c r="F237" t="s">
+      <c r="F237" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G237" s="1" t="s">
@@ -6330,7 +6415,7 @@
     </row>
     <row r="238" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A238" s="1">
-        <v>257</v>
+        <v>237</v>
       </c>
       <c r="B238" s="1" t="s">
         <v>150</v>
@@ -6344,7 +6429,7 @@
       <c r="E238" s="2">
         <v>10589643004</v>
       </c>
-      <c r="F238" t="s">
+      <c r="F238" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G238" s="1" t="s">
@@ -6353,7 +6438,7 @@
     </row>
     <row r="239" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A239" s="1">
-        <v>258</v>
+        <v>238</v>
       </c>
       <c r="B239" s="1" t="s">
         <v>150</v>
@@ -6367,7 +6452,7 @@
       <c r="E239" s="2">
         <v>3252244500</v>
       </c>
-      <c r="F239" t="s">
+      <c r="F239" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G239" s="1" t="s">
@@ -6376,7 +6461,7 @@
     </row>
     <row r="240" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A240" s="1">
-        <v>259</v>
+        <v>239</v>
       </c>
       <c r="B240" s="1" t="s">
         <v>150</v>
@@ -6390,7 +6475,7 @@
       <c r="E240" s="2">
         <v>4191108684</v>
       </c>
-      <c r="F240" t="s">
+      <c r="F240" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G240" s="1" t="s">
@@ -6399,7 +6484,7 @@
     </row>
     <row r="241" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A241" s="1">
-        <v>260</v>
+        <v>240</v>
       </c>
       <c r="B241" s="1" t="s">
         <v>150</v>
@@ -6413,7 +6498,7 @@
       <c r="E241" s="2">
         <v>4937711997</v>
       </c>
-      <c r="F241" t="s">
+      <c r="F241" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G241" s="1" t="s">
@@ -6422,7 +6507,7 @@
     </row>
     <row r="242" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A242" s="1">
-        <v>261</v>
+        <v>241</v>
       </c>
       <c r="B242" s="1" t="s">
         <v>150</v>
@@ -6436,11 +6521,471 @@
       <c r="E242" s="2">
         <v>160708941019</v>
       </c>
-      <c r="F242" t="s">
+      <c r="F242" s="5" t="s">
         <v>153</v>
       </c>
       <c r="G242" s="1" t="s">
         <v>162</v>
+      </c>
+    </row>
+    <row r="243" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A243" s="1">
+        <v>242</v>
+      </c>
+      <c r="B243" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C243" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D243" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="E243" s="2">
+        <v>6000</v>
+      </c>
+      <c r="F243" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G243" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="244" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A244" s="1">
+        <v>243</v>
+      </c>
+      <c r="B244" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C244" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D244" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E244" s="2">
+        <v>4500</v>
+      </c>
+      <c r="F244" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G244" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="245" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A245" s="1">
+        <v>244</v>
+      </c>
+      <c r="B245" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C245" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D245" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="E245" s="6">
+        <v>44500</v>
+      </c>
+      <c r="F245" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G245" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="246" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A246" s="1">
+        <v>245</v>
+      </c>
+      <c r="B246" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C246" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D246" s="5" t="s">
+        <v>170</v>
+      </c>
+      <c r="E246" s="6">
+        <v>73000</v>
+      </c>
+      <c r="F246" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G246" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="247" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A247" s="1">
+        <v>246</v>
+      </c>
+      <c r="B247" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C247" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D247" s="5" t="s">
+        <v>171</v>
+      </c>
+      <c r="E247" s="6">
+        <v>71000</v>
+      </c>
+      <c r="F247" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G247" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="248" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A248" s="1">
+        <v>247</v>
+      </c>
+      <c r="B248" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C248" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D248" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="E248" s="6">
+        <v>1164000</v>
+      </c>
+      <c r="F248" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G248" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="249" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A249" s="1">
+        <v>248</v>
+      </c>
+      <c r="B249" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C249" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D249" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="E249" s="6">
+        <v>84500</v>
+      </c>
+      <c r="F249" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G249" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="250" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A250" s="1">
+        <v>249</v>
+      </c>
+      <c r="B250" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C250" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D250" s="5" t="s">
+        <v>174</v>
+      </c>
+      <c r="E250" s="6">
+        <v>691000</v>
+      </c>
+      <c r="F250" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G250" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="251" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A251" s="1">
+        <v>250</v>
+      </c>
+      <c r="B251" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C251" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D251" s="5" t="s">
+        <v>175</v>
+      </c>
+      <c r="E251" s="6">
+        <v>92500</v>
+      </c>
+      <c r="F251" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G251" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="252" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A252" s="1">
+        <v>251</v>
+      </c>
+      <c r="B252" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C252" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D252" s="5" t="s">
+        <v>176</v>
+      </c>
+      <c r="E252" s="6">
+        <v>22500</v>
+      </c>
+      <c r="F252" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G252" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="253" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A253" s="1">
+        <v>252</v>
+      </c>
+      <c r="B253" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C253" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D253" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="E253" s="6">
+        <v>16000</v>
+      </c>
+      <c r="F253" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G253" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="254" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A254" s="1">
+        <v>253</v>
+      </c>
+      <c r="B254" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C254" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D254" s="5" t="s">
+        <v>178</v>
+      </c>
+      <c r="E254" s="6">
+        <v>37000</v>
+      </c>
+      <c r="F254" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G254" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="255" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A255" s="1">
+        <v>254</v>
+      </c>
+      <c r="B255" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C255" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D255" s="5" t="s">
+        <v>179</v>
+      </c>
+      <c r="E255" s="6">
+        <v>10000</v>
+      </c>
+      <c r="F255" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G255" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="256" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A256" s="1">
+        <v>255</v>
+      </c>
+      <c r="B256" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C256" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D256" s="5" t="s">
+        <v>180</v>
+      </c>
+      <c r="E256" s="6">
+        <v>30000</v>
+      </c>
+      <c r="F256" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G256" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="257" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A257" s="1">
+        <v>256</v>
+      </c>
+      <c r="B257" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C257" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D257" s="5" t="s">
+        <v>181</v>
+      </c>
+      <c r="E257" s="6">
+        <v>70000</v>
+      </c>
+      <c r="F257" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G257" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="258" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A258" s="1">
+        <v>257</v>
+      </c>
+      <c r="B258" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C258" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D258" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="E258" s="6">
+        <v>39000</v>
+      </c>
+      <c r="F258" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G258" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="259" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A259" s="1">
+        <v>258</v>
+      </c>
+      <c r="B259" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C259" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D259" s="5" t="s">
+        <v>183</v>
+      </c>
+      <c r="E259" s="6">
+        <v>22500</v>
+      </c>
+      <c r="F259" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G259" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="260" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A260" s="1">
+        <v>259</v>
+      </c>
+      <c r="B260" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C260" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D260" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="E260" s="6">
+        <v>220000</v>
+      </c>
+      <c r="F260" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G260" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="261" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A261" s="1">
+        <v>260</v>
+      </c>
+      <c r="B261" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C261" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="D261" s="5" t="s">
+        <v>185</v>
+      </c>
+      <c r="E261" s="6">
+        <v>710000</v>
+      </c>
+      <c r="F261" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G261" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="262" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A262" s="1">
+        <v>261</v>
+      </c>
+      <c r="B262" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="C262" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="D262" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="E262" s="7">
+        <v>3408000</v>
+      </c>
+      <c r="F262" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="G262" s="1" t="s">
+        <v>156</v>
       </c>
     </row>
   </sheetData>

</xml_diff>